<commit_message>
Add Lancaster 2017 + 2019 primaries
Same hierarchical HTML site (vr.co.lancaster.pa.us), parsed by the
existing LancasterHtmlSource. Pre-2021 archives have smaller coverage
(2019 walks 26 race pages; 2023 walked 435), reflecting either a
sparser local-race archive or fewer multi-candidate primaries that
year. Zero new RCV-useful races surface from either year — most
contests are uncontested or have a clear majority winner.

Top_RCV_Races: 184 -> 185.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Top_RCV_Races.xlsx
+++ b/Top_RCV_Races.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3376" uniqueCount="918">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3384" uniqueCount="923">
   <si>
     <t>Year</t>
   </si>
@@ -2371,6 +2371,9 @@
     <t>REP Supervisor Zerbe Township</t>
   </si>
   <si>
+    <t>SUPERVISOR LIGONIER TOWNSHIP</t>
+  </si>
+  <si>
     <t>REP SUPERVISOR UPPER YODER TOWNSHIP</t>
   </si>
   <si>
@@ -2470,6 +2473,9 @@
     <t>DANIEL TUBBY BILLIG</t>
   </si>
   <si>
+    <t>REP ERIK ROSS</t>
+  </si>
+  <si>
     <t>SUE KONVOLINKA</t>
   </si>
   <si>
@@ -2560,6 +2566,9 @@
     <t>WALTER PACZKOSKIE</t>
   </si>
   <si>
+    <t>REP DANIEL RESENIC</t>
+  </si>
+  <si>
     <t>KYLE SHAFFER</t>
   </si>
   <si>
@@ -2647,6 +2656,9 @@
     <t>MIKE SCHWARTZ</t>
   </si>
   <si>
+    <t>DEM ROXANNE SHADRON</t>
+  </si>
+  <si>
     <t>BOB VARNER</t>
   </si>
   <si>
@@ -2741,6 +2753,9 @@
   </si>
   <si>
     <t>DANIEL TUBBY BILLIG 45.3%, WALTER PACZKOSKIE 27.8%, MIKE SCHWARTZ 26.8%</t>
+  </si>
+  <si>
+    <t>REP ERIK ROSS 43.9%, REP DANIEL RESENIC 35.3%, DEM ROXANNE SHADRON 20.7%</t>
   </si>
   <si>
     <t>SUE KONVOLINKA 44.0%, KYLE SHAFFER 23.5%, BOB VARNER 17.5%, JEFFREY MASTERSON 8.1%, BOB AMISTADI 7.0%</t>
@@ -13442,7 +13457,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N185"/>
+  <dimension ref="A1:N186"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -13773,13 +13788,13 @@
         <v>4</v>
       </c>
       <c r="G8" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="H8">
         <v>41.98</v>
       </c>
       <c r="I8" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="J8">
         <v>29.23</v>
@@ -13794,7 +13809,7 @@
         <v>12.75</v>
       </c>
       <c r="N8" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -13949,19 +13964,19 @@
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="H12">
         <v>44.49</v>
       </c>
       <c r="I12" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="J12">
         <v>29.78</v>
       </c>
       <c r="K12" t="s">
-        <v>856</v>
+        <v>859</v>
       </c>
       <c r="L12">
         <v>25.74</v>
@@ -13970,7 +13985,7 @@
         <v>14.71</v>
       </c>
       <c r="N12" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -14081,19 +14096,19 @@
         <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="H15">
         <v>41.68</v>
       </c>
       <c r="I15" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="J15">
         <v>30.54</v>
       </c>
       <c r="K15" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="L15">
         <v>27.78</v>
@@ -14102,7 +14117,7 @@
         <v>11.14</v>
       </c>
       <c r="N15" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -14609,19 +14624,19 @@
         <v>3</v>
       </c>
       <c r="G27" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="H27">
         <v>43.21</v>
       </c>
       <c r="I27" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="J27">
         <v>29.8</v>
       </c>
       <c r="K27" t="s">
-        <v>857</v>
+        <v>860</v>
       </c>
       <c r="L27">
         <v>27</v>
@@ -14630,7 +14645,7 @@
         <v>13.41</v>
       </c>
       <c r="N27" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -15181,19 +15196,19 @@
         <v>5</v>
       </c>
       <c r="G40" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="H40">
         <v>41.6</v>
       </c>
       <c r="I40" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="J40">
         <v>25.18</v>
       </c>
       <c r="K40" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="L40">
         <v>16.75</v>
@@ -15202,7 +15217,7 @@
         <v>16.42</v>
       </c>
       <c r="N40" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -15313,19 +15328,19 @@
         <v>4</v>
       </c>
       <c r="G43" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="H43">
         <v>46.5</v>
       </c>
       <c r="I43" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="J43">
         <v>27.04</v>
       </c>
       <c r="K43" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="L43">
         <v>13.38</v>
@@ -15334,7 +15349,7 @@
         <v>19.45</v>
       </c>
       <c r="N43" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -15445,19 +15460,19 @@
         <v>4</v>
       </c>
       <c r="G46" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="H46">
         <v>42.2</v>
       </c>
       <c r="I46" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="J46">
         <v>35.81</v>
       </c>
       <c r="K46" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="L46">
         <v>14.91</v>
@@ -15466,7 +15481,7 @@
         <v>6.39</v>
       </c>
       <c r="N46" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -15533,19 +15548,19 @@
         <v>3</v>
       </c>
       <c r="G48" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="H48">
         <v>46.08</v>
       </c>
       <c r="I48" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="J48">
         <v>27.29</v>
       </c>
       <c r="K48" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="L48">
         <v>26.63</v>
@@ -15554,7 +15569,7 @@
         <v>18.79</v>
       </c>
       <c r="N48" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -15577,19 +15592,19 @@
         <v>4</v>
       </c>
       <c r="G49" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="H49">
         <v>47.47</v>
       </c>
       <c r="I49" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="J49">
         <v>24.83</v>
       </c>
       <c r="K49" t="s">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="L49">
         <v>23.46</v>
@@ -15598,7 +15613,7 @@
         <v>22.63</v>
       </c>
       <c r="N49" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -15621,19 +15636,19 @@
         <v>4</v>
       </c>
       <c r="G50" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="H50">
         <v>44.12</v>
       </c>
       <c r="I50" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="J50">
         <v>24.37</v>
       </c>
       <c r="K50" t="s">
-        <v>863</v>
+        <v>866</v>
       </c>
       <c r="L50">
         <v>21.33</v>
@@ -15642,7 +15657,7 @@
         <v>19.75</v>
       </c>
       <c r="N50" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
     </row>
     <row r="51" spans="1:14">
@@ -15753,19 +15768,19 @@
         <v>3</v>
       </c>
       <c r="G53" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="H53">
         <v>49.43</v>
       </c>
       <c r="I53" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="J53">
         <v>44.1</v>
       </c>
       <c r="K53" t="s">
-        <v>864</v>
+        <v>867</v>
       </c>
       <c r="L53">
         <v>6.47</v>
@@ -15774,7 +15789,7 @@
         <v>5.33</v>
       </c>
       <c r="N53" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -15929,13 +15944,13 @@
         <v>6</v>
       </c>
       <c r="G57" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="H57">
         <v>40.4</v>
       </c>
       <c r="I57" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="J57">
         <v>25.88</v>
@@ -15950,7 +15965,7 @@
         <v>14.52</v>
       </c>
       <c r="N57" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -16369,19 +16384,19 @@
         <v>3</v>
       </c>
       <c r="G67" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="H67">
         <v>38.37</v>
       </c>
       <c r="I67" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="J67">
         <v>31.83</v>
       </c>
       <c r="K67" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="L67">
         <v>29.81</v>
@@ -16390,7 +16405,7 @@
         <v>6.54</v>
       </c>
       <c r="N67" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -16677,19 +16692,19 @@
         <v>3</v>
       </c>
       <c r="G74" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="H74">
         <v>48.83</v>
       </c>
       <c r="I74" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="J74">
         <v>39.89</v>
       </c>
       <c r="K74" t="s">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="L74">
         <v>11.28</v>
@@ -16698,7 +16713,7 @@
         <v>8.949999999999999</v>
       </c>
       <c r="N74" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -16765,19 +16780,19 @@
         <v>3</v>
       </c>
       <c r="G76" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="H76">
         <v>41.34</v>
       </c>
       <c r="I76" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="J76">
         <v>33.12</v>
       </c>
       <c r="K76" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="L76">
         <v>25.54</v>
@@ -16786,7 +16801,7 @@
         <v>8.210000000000001</v>
       </c>
       <c r="N76" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -17205,19 +17220,19 @@
         <v>4</v>
       </c>
       <c r="G86" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="H86">
         <v>49.36</v>
       </c>
       <c r="I86" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="J86">
         <v>22.31</v>
       </c>
       <c r="K86" t="s">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="L86">
         <v>14.32</v>
@@ -17226,7 +17241,7 @@
         <v>27.06</v>
       </c>
       <c r="N86" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -17909,19 +17924,19 @@
         <v>3</v>
       </c>
       <c r="G102" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="H102">
         <v>44.61</v>
       </c>
       <c r="I102" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="J102">
         <v>34.43</v>
       </c>
       <c r="K102" t="s">
-        <v>869</v>
+        <v>872</v>
       </c>
       <c r="L102">
         <v>20.96</v>
@@ -17930,7 +17945,7 @@
         <v>10.18</v>
       </c>
       <c r="N102" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -18173,19 +18188,19 @@
         <v>3</v>
       </c>
       <c r="G108" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="H108">
         <v>48.84</v>
       </c>
       <c r="I108" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
       <c r="J108">
         <v>31.48</v>
       </c>
       <c r="K108" t="s">
-        <v>870</v>
+        <v>873</v>
       </c>
       <c r="L108">
         <v>19.68</v>
@@ -18194,7 +18209,7 @@
         <v>17.36</v>
       </c>
       <c r="N108" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -18217,7 +18232,7 @@
         <v>3</v>
       </c>
       <c r="G109" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="H109">
         <v>48.33</v>
@@ -18229,7 +18244,7 @@
         <v>30.65</v>
       </c>
       <c r="K109" t="s">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="L109">
         <v>21.02</v>
@@ -18238,7 +18253,7 @@
         <v>17.69</v>
       </c>
       <c r="N109" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -18305,19 +18320,19 @@
         <v>3</v>
       </c>
       <c r="G111" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="H111">
         <v>47.43</v>
       </c>
       <c r="I111" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
       <c r="J111">
         <v>26.52</v>
       </c>
       <c r="K111" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
       <c r="L111">
         <v>26.04</v>
@@ -18326,7 +18341,7 @@
         <v>20.91</v>
       </c>
       <c r="N111" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -18349,19 +18364,19 @@
         <v>4</v>
       </c>
       <c r="G112" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="H112">
         <v>47.32</v>
       </c>
       <c r="I112" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="J112">
         <v>36.47</v>
       </c>
       <c r="K112" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
       <c r="L112">
         <v>8.57</v>
@@ -18370,7 +18385,7 @@
         <v>10.84</v>
       </c>
       <c r="N112" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
     </row>
     <row r="113" spans="1:14">
@@ -18613,19 +18628,19 @@
         <v>4</v>
       </c>
       <c r="G118" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="H118">
         <v>41.39</v>
       </c>
       <c r="I118" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="J118">
         <v>31.39</v>
       </c>
       <c r="K118" t="s">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="L118">
         <v>16.39</v>
@@ -18634,7 +18649,7 @@
         <v>10</v>
       </c>
       <c r="N118" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
     </row>
     <row r="119" spans="1:14">
@@ -18657,19 +18672,19 @@
         <v>3</v>
       </c>
       <c r="G119" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="H119">
         <v>45.32</v>
       </c>
       <c r="I119" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
       <c r="J119">
         <v>27.85</v>
       </c>
       <c r="K119" t="s">
-        <v>875</v>
+        <v>878</v>
       </c>
       <c r="L119">
         <v>26.84</v>
@@ -18678,7 +18693,7 @@
         <v>17.47</v>
       </c>
       <c r="N119" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
     </row>
     <row r="120" spans="1:14">
@@ -18771,46 +18786,46 @@
     </row>
     <row r="122" spans="1:14">
       <c r="A122">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B122" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C122" t="s">
         <v>17</v>
       </c>
       <c r="D122" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E122" t="s">
-        <v>69</v>
+        <v>784</v>
       </c>
       <c r="F122">
         <v>3</v>
       </c>
       <c r="G122" t="s">
-        <v>134</v>
+        <v>818</v>
       </c>
       <c r="H122">
-        <v>38.95</v>
+        <v>43.93</v>
       </c>
       <c r="I122" t="s">
-        <v>197</v>
+        <v>849</v>
       </c>
       <c r="J122">
-        <v>37.45</v>
+        <v>35.35</v>
       </c>
       <c r="K122" t="s">
-        <v>260</v>
+        <v>879</v>
       </c>
       <c r="L122">
-        <v>23.6</v>
+        <v>20.72</v>
       </c>
       <c r="M122">
-        <v>1.5</v>
+        <v>8.58</v>
       </c>
       <c r="N122" t="s">
-        <v>325</v>
+        <v>912</v>
       </c>
     </row>
     <row r="123" spans="1:14">
@@ -18824,37 +18839,37 @@
         <v>17</v>
       </c>
       <c r="D123" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E123" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="F123">
         <v>3</v>
       </c>
       <c r="G123" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="H123">
-        <v>37.08</v>
+        <v>38.95</v>
       </c>
       <c r="I123" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="J123">
-        <v>34.47</v>
+        <v>37.45</v>
       </c>
       <c r="K123" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="L123">
-        <v>28.44</v>
+        <v>23.6</v>
       </c>
       <c r="M123">
-        <v>2.61</v>
+        <v>1.5</v>
       </c>
       <c r="N123" t="s">
-        <v>341</v>
+        <v>325</v>
       </c>
     </row>
     <row r="124" spans="1:14">
@@ -18868,37 +18883,37 @@
         <v>17</v>
       </c>
       <c r="D124" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E124" t="s">
-        <v>511</v>
+        <v>85</v>
       </c>
       <c r="F124">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G124" t="s">
-        <v>569</v>
+        <v>149</v>
       </c>
       <c r="H124">
-        <v>45.6</v>
+        <v>37.08</v>
       </c>
       <c r="I124" t="s">
-        <v>618</v>
+        <v>213</v>
       </c>
       <c r="J124">
-        <v>25.96</v>
+        <v>34.47</v>
       </c>
       <c r="K124" t="s">
-        <v>635</v>
+        <v>276</v>
       </c>
       <c r="L124">
-        <v>20.63</v>
+        <v>28.44</v>
       </c>
       <c r="M124">
-        <v>19.65</v>
+        <v>2.61</v>
       </c>
       <c r="N124" t="s">
-        <v>727</v>
+        <v>341</v>
       </c>
     </row>
     <row r="125" spans="1:14">
@@ -18912,37 +18927,37 @@
         <v>17</v>
       </c>
       <c r="D125" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E125" t="s">
-        <v>391</v>
+        <v>511</v>
       </c>
       <c r="F125">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G125" t="s">
-        <v>129</v>
+        <v>569</v>
       </c>
       <c r="H125">
-        <v>39.99</v>
+        <v>45.6</v>
       </c>
       <c r="I125" t="s">
-        <v>256</v>
+        <v>618</v>
       </c>
       <c r="J125">
-        <v>25.8</v>
+        <v>25.96</v>
       </c>
       <c r="K125" t="s">
-        <v>455</v>
+        <v>635</v>
       </c>
       <c r="L125">
-        <v>18.52</v>
+        <v>20.63</v>
       </c>
       <c r="M125">
-        <v>14.19</v>
+        <v>19.65</v>
       </c>
       <c r="N125" t="s">
-        <v>480</v>
+        <v>727</v>
       </c>
     </row>
     <row r="126" spans="1:14">
@@ -18956,37 +18971,37 @@
         <v>17</v>
       </c>
       <c r="D126" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E126" t="s">
-        <v>502</v>
+        <v>391</v>
       </c>
       <c r="F126">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G126" t="s">
-        <v>560</v>
+        <v>129</v>
       </c>
       <c r="H126">
-        <v>43.29</v>
+        <v>39.99</v>
       </c>
       <c r="I126" t="s">
-        <v>610</v>
+        <v>256</v>
       </c>
       <c r="J126">
-        <v>34.34</v>
+        <v>25.8</v>
       </c>
       <c r="K126" t="s">
-        <v>665</v>
+        <v>455</v>
       </c>
       <c r="L126">
-        <v>22.37</v>
+        <v>18.52</v>
       </c>
       <c r="M126">
-        <v>8.949999999999999</v>
+        <v>14.19</v>
       </c>
       <c r="N126" t="s">
-        <v>718</v>
+        <v>480</v>
       </c>
     </row>
     <row r="127" spans="1:14">
@@ -19003,34 +19018,34 @@
         <v>27</v>
       </c>
       <c r="E127" t="s">
-        <v>522</v>
+        <v>502</v>
       </c>
       <c r="F127">
         <v>3</v>
       </c>
       <c r="G127" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="H127">
-        <v>46.95</v>
+        <v>43.29</v>
       </c>
       <c r="I127" t="s">
-        <v>629</v>
+        <v>610</v>
       </c>
       <c r="J127">
-        <v>27.11</v>
+        <v>34.34</v>
       </c>
       <c r="K127" t="s">
-        <v>616</v>
+        <v>665</v>
       </c>
       <c r="L127">
-        <v>25.94</v>
+        <v>22.37</v>
       </c>
       <c r="M127">
-        <v>19.84</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="N127" t="s">
-        <v>738</v>
+        <v>718</v>
       </c>
     </row>
     <row r="128" spans="1:14">
@@ -19044,37 +19059,37 @@
         <v>17</v>
       </c>
       <c r="D128" t="s">
-        <v>366</v>
+        <v>27</v>
       </c>
       <c r="E128" t="s">
-        <v>380</v>
+        <v>522</v>
       </c>
       <c r="F128">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G128" t="s">
-        <v>404</v>
+        <v>566</v>
       </c>
       <c r="H128">
-        <v>36.72</v>
+        <v>46.95</v>
       </c>
       <c r="I128" t="s">
-        <v>426</v>
+        <v>629</v>
       </c>
       <c r="J128">
-        <v>23.24</v>
+        <v>27.11</v>
       </c>
       <c r="K128" t="s">
-        <v>447</v>
+        <v>616</v>
       </c>
       <c r="L128">
-        <v>21.51</v>
+        <v>25.94</v>
       </c>
       <c r="M128">
-        <v>13.48</v>
+        <v>19.84</v>
       </c>
       <c r="N128" t="s">
-        <v>469</v>
+        <v>738</v>
       </c>
     </row>
     <row r="129" spans="1:14">
@@ -19088,37 +19103,37 @@
         <v>17</v>
       </c>
       <c r="D129" t="s">
-        <v>30</v>
+        <v>366</v>
       </c>
       <c r="E129" t="s">
-        <v>505</v>
+        <v>380</v>
       </c>
       <c r="F129">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G129" t="s">
-        <v>563</v>
+        <v>404</v>
       </c>
       <c r="H129">
-        <v>43.91</v>
+        <v>36.72</v>
       </c>
       <c r="I129" t="s">
-        <v>613</v>
+        <v>426</v>
       </c>
       <c r="J129">
-        <v>29.17</v>
+        <v>23.24</v>
       </c>
       <c r="K129" t="s">
-        <v>668</v>
+        <v>447</v>
       </c>
       <c r="L129">
-        <v>26.92</v>
+        <v>21.51</v>
       </c>
       <c r="M129">
-        <v>14.74</v>
+        <v>13.48</v>
       </c>
       <c r="N129" t="s">
-        <v>721</v>
+        <v>469</v>
       </c>
     </row>
     <row r="130" spans="1:14">
@@ -19135,34 +19150,34 @@
         <v>30</v>
       </c>
       <c r="E130" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="F130">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G130" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="H130">
-        <v>45.68</v>
+        <v>43.91</v>
       </c>
       <c r="I130" t="s">
-        <v>619</v>
+        <v>613</v>
       </c>
       <c r="J130">
-        <v>21.47</v>
+        <v>29.17</v>
       </c>
       <c r="K130" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="L130">
-        <v>17.72</v>
+        <v>26.92</v>
       </c>
       <c r="M130">
-        <v>24.21</v>
+        <v>14.74</v>
       </c>
       <c r="N130" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
     </row>
     <row r="131" spans="1:14">
@@ -19176,37 +19191,37 @@
         <v>17</v>
       </c>
       <c r="D131" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E131" t="s">
-        <v>386</v>
+        <v>512</v>
       </c>
       <c r="F131">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G131" t="s">
-        <v>233</v>
+        <v>570</v>
       </c>
       <c r="H131">
-        <v>38.33</v>
+        <v>45.68</v>
       </c>
       <c r="I131" t="s">
-        <v>169</v>
+        <v>619</v>
       </c>
       <c r="J131">
-        <v>18.9</v>
+        <v>21.47</v>
       </c>
       <c r="K131" t="s">
-        <v>297</v>
+        <v>672</v>
       </c>
       <c r="L131">
-        <v>17.73</v>
+        <v>17.72</v>
       </c>
       <c r="M131">
-        <v>19.43</v>
+        <v>24.21</v>
       </c>
       <c r="N131" t="s">
-        <v>475</v>
+        <v>728</v>
       </c>
     </row>
     <row r="132" spans="1:14">
@@ -19220,37 +19235,37 @@
         <v>17</v>
       </c>
       <c r="D132" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E132" t="s">
-        <v>70</v>
+        <v>386</v>
       </c>
       <c r="F132">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G132" t="s">
-        <v>135</v>
+        <v>233</v>
       </c>
       <c r="H132">
-        <v>36.62</v>
+        <v>38.33</v>
       </c>
       <c r="I132" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="J132">
-        <v>35.09</v>
+        <v>18.9</v>
       </c>
       <c r="K132" t="s">
-        <v>261</v>
+        <v>297</v>
       </c>
       <c r="L132">
-        <v>28.28</v>
+        <v>17.73</v>
       </c>
       <c r="M132">
-        <v>1.53</v>
+        <v>19.43</v>
       </c>
       <c r="N132" t="s">
-        <v>326</v>
+        <v>475</v>
       </c>
     </row>
     <row r="133" spans="1:14">
@@ -19264,37 +19279,37 @@
         <v>17</v>
       </c>
       <c r="D133" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E133" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="F133">
         <v>3</v>
       </c>
       <c r="G133" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="H133">
-        <v>34.01</v>
+        <v>36.62</v>
       </c>
       <c r="I133" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="J133">
-        <v>33.39</v>
+        <v>35.09</v>
       </c>
       <c r="K133" t="s">
-        <v>244</v>
+        <v>261</v>
       </c>
       <c r="L133">
-        <v>32.6</v>
+        <v>28.28</v>
       </c>
       <c r="M133">
-        <v>0.61</v>
+        <v>1.53</v>
       </c>
       <c r="N133" t="s">
-        <v>308</v>
+        <v>326</v>
       </c>
     </row>
     <row r="134" spans="1:14">
@@ -19308,37 +19323,37 @@
         <v>17</v>
       </c>
       <c r="D134" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E134" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F134">
         <v>3</v>
       </c>
       <c r="G134" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H134">
-        <v>46.2</v>
+        <v>34.01</v>
       </c>
       <c r="I134" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="J134">
-        <v>45.92</v>
+        <v>33.39</v>
       </c>
       <c r="K134" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="L134">
-        <v>7.88</v>
+        <v>32.6</v>
       </c>
       <c r="M134">
-        <v>0.27</v>
+        <v>0.61</v>
       </c>
       <c r="N134" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
     </row>
     <row r="135" spans="1:14">
@@ -19352,37 +19367,37 @@
         <v>17</v>
       </c>
       <c r="D135" t="s">
-        <v>481</v>
+        <v>21</v>
       </c>
       <c r="E135" t="s">
-        <v>530</v>
+        <v>46</v>
       </c>
       <c r="F135">
         <v>3</v>
       </c>
       <c r="G135" t="s">
-        <v>583</v>
+        <v>111</v>
       </c>
       <c r="H135">
-        <v>47.82</v>
+        <v>46.2</v>
       </c>
       <c r="I135" t="s">
-        <v>636</v>
+        <v>174</v>
       </c>
       <c r="J135">
-        <v>27.86</v>
+        <v>45.92</v>
       </c>
       <c r="K135" t="s">
-        <v>687</v>
+        <v>238</v>
       </c>
       <c r="L135">
-        <v>24.32</v>
+        <v>7.88</v>
       </c>
       <c r="M135">
-        <v>19.96</v>
+        <v>0.27</v>
       </c>
       <c r="N135" t="s">
-        <v>747</v>
+        <v>302</v>
       </c>
     </row>
     <row r="136" spans="1:14">
@@ -19396,37 +19411,37 @@
         <v>17</v>
       </c>
       <c r="D136" t="s">
-        <v>40</v>
+        <v>481</v>
       </c>
       <c r="E136" t="s">
-        <v>535</v>
+        <v>530</v>
       </c>
       <c r="F136">
         <v>3</v>
       </c>
       <c r="G136" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="H136">
-        <v>48.85</v>
+        <v>47.82</v>
       </c>
       <c r="I136" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
       <c r="J136">
-        <v>42.35</v>
+        <v>27.86</v>
       </c>
       <c r="K136" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
       <c r="L136">
-        <v>8.800000000000001</v>
+        <v>24.32</v>
       </c>
       <c r="M136">
-        <v>6.5</v>
+        <v>19.96</v>
       </c>
       <c r="N136" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
     </row>
     <row r="137" spans="1:14">
@@ -19440,37 +19455,37 @@
         <v>17</v>
       </c>
       <c r="D137" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E137" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="F137">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G137" t="s">
-        <v>569</v>
+        <v>588</v>
       </c>
       <c r="H137">
-        <v>47.79</v>
+        <v>48.85</v>
       </c>
       <c r="I137" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="J137">
-        <v>27.76</v>
+        <v>42.35</v>
       </c>
       <c r="K137" t="s">
-        <v>618</v>
+        <v>692</v>
       </c>
       <c r="L137">
-        <v>15.83</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M137">
-        <v>20.03</v>
+        <v>6.5</v>
       </c>
       <c r="N137" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
     </row>
     <row r="138" spans="1:14">
@@ -19484,37 +19499,37 @@
         <v>17</v>
       </c>
       <c r="D138" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E138" t="s">
-        <v>64</v>
+        <v>529</v>
       </c>
       <c r="F138">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G138" t="s">
-        <v>129</v>
+        <v>569</v>
       </c>
       <c r="H138">
-        <v>32.53</v>
+        <v>47.79</v>
       </c>
       <c r="I138" t="s">
-        <v>192</v>
+        <v>635</v>
       </c>
       <c r="J138">
-        <v>31.37</v>
+        <v>27.76</v>
       </c>
       <c r="K138" t="s">
-        <v>256</v>
+        <v>618</v>
       </c>
       <c r="L138">
-        <v>17.8</v>
+        <v>15.83</v>
       </c>
       <c r="M138">
-        <v>1.15</v>
+        <v>20.03</v>
       </c>
       <c r="N138" t="s">
-        <v>320</v>
+        <v>746</v>
       </c>
     </row>
     <row r="139" spans="1:14">
@@ -19528,37 +19543,37 @@
         <v>17</v>
       </c>
       <c r="D139" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E139" t="s">
-        <v>536</v>
+        <v>64</v>
       </c>
       <c r="F139">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G139" t="s">
-        <v>560</v>
+        <v>129</v>
       </c>
       <c r="H139">
-        <v>48.87</v>
+        <v>32.53</v>
       </c>
       <c r="I139" t="s">
-        <v>610</v>
+        <v>192</v>
       </c>
       <c r="J139">
-        <v>38.55</v>
+        <v>31.37</v>
       </c>
       <c r="K139" t="s">
-        <v>665</v>
+        <v>256</v>
       </c>
       <c r="L139">
-        <v>12.58</v>
+        <v>17.8</v>
       </c>
       <c r="M139">
-        <v>10.31</v>
+        <v>1.15</v>
       </c>
       <c r="N139" t="s">
-        <v>753</v>
+        <v>320</v>
       </c>
     </row>
     <row r="140" spans="1:14">
@@ -19575,34 +19590,34 @@
         <v>27</v>
       </c>
       <c r="E140" t="s">
-        <v>508</v>
+        <v>536</v>
       </c>
       <c r="F140">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G140" t="s">
-        <v>566</v>
+        <v>560</v>
       </c>
       <c r="H140">
-        <v>44.46</v>
+        <v>48.87</v>
       </c>
       <c r="I140" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="J140">
-        <v>28.34</v>
+        <v>38.55</v>
       </c>
       <c r="K140" t="s">
-        <v>629</v>
+        <v>665</v>
       </c>
       <c r="L140">
-        <v>22.18</v>
+        <v>12.58</v>
       </c>
       <c r="M140">
-        <v>16.12</v>
+        <v>10.31</v>
       </c>
       <c r="N140" t="s">
-        <v>724</v>
+        <v>753</v>
       </c>
     </row>
     <row r="141" spans="1:14">
@@ -19616,37 +19631,37 @@
         <v>17</v>
       </c>
       <c r="D141" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="E141" t="s">
-        <v>77</v>
+        <v>508</v>
       </c>
       <c r="F141">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G141" t="s">
-        <v>141</v>
+        <v>566</v>
       </c>
       <c r="H141">
-        <v>46.38</v>
+        <v>44.46</v>
       </c>
       <c r="I141" t="s">
-        <v>205</v>
+        <v>616</v>
       </c>
       <c r="J141">
-        <v>44.44</v>
+        <v>28.34</v>
       </c>
       <c r="K141" t="s">
-        <v>268</v>
+        <v>629</v>
       </c>
       <c r="L141">
-        <v>9.18</v>
+        <v>22.18</v>
       </c>
       <c r="M141">
-        <v>1.95</v>
+        <v>16.12</v>
       </c>
       <c r="N141" t="s">
-        <v>333</v>
+        <v>724</v>
       </c>
     </row>
     <row r="142" spans="1:14">
@@ -19660,37 +19675,37 @@
         <v>17</v>
       </c>
       <c r="D142" t="s">
-        <v>366</v>
+        <v>37</v>
       </c>
       <c r="E142" t="s">
-        <v>501</v>
+        <v>77</v>
       </c>
       <c r="F142">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G142" t="s">
-        <v>559</v>
+        <v>141</v>
       </c>
       <c r="H142">
-        <v>43.13</v>
+        <v>46.38</v>
       </c>
       <c r="I142" t="s">
-        <v>426</v>
+        <v>205</v>
       </c>
       <c r="J142">
-        <v>26.27</v>
+        <v>44.44</v>
       </c>
       <c r="K142" t="s">
-        <v>447</v>
+        <v>268</v>
       </c>
       <c r="L142">
-        <v>19.77</v>
+        <v>9.18</v>
       </c>
       <c r="M142">
-        <v>16.86</v>
+        <v>1.95</v>
       </c>
       <c r="N142" t="s">
-        <v>717</v>
+        <v>333</v>
       </c>
     </row>
     <row r="143" spans="1:14">
@@ -19704,37 +19719,37 @@
         <v>17</v>
       </c>
       <c r="D143" t="s">
-        <v>30</v>
+        <v>366</v>
       </c>
       <c r="E143" t="s">
-        <v>518</v>
+        <v>501</v>
       </c>
       <c r="F143">
         <v>5</v>
       </c>
       <c r="G143" t="s">
-        <v>570</v>
+        <v>559</v>
       </c>
       <c r="H143">
-        <v>46.48</v>
+        <v>43.13</v>
       </c>
       <c r="I143" t="s">
-        <v>625</v>
+        <v>426</v>
       </c>
       <c r="J143">
-        <v>18.62</v>
+        <v>26.27</v>
       </c>
       <c r="K143" t="s">
-        <v>677</v>
+        <v>447</v>
       </c>
       <c r="L143">
-        <v>14.39</v>
+        <v>19.77</v>
       </c>
       <c r="M143">
-        <v>27.85</v>
+        <v>16.86</v>
       </c>
       <c r="N143" t="s">
-        <v>734</v>
+        <v>717</v>
       </c>
     </row>
     <row r="144" spans="1:14">
@@ -19751,34 +19766,34 @@
         <v>30</v>
       </c>
       <c r="E144" t="s">
-        <v>79</v>
+        <v>518</v>
       </c>
       <c r="F144">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G144" t="s">
-        <v>143</v>
+        <v>570</v>
       </c>
       <c r="H144">
-        <v>42.6</v>
+        <v>46.48</v>
       </c>
       <c r="I144" t="s">
-        <v>207</v>
+        <v>625</v>
       </c>
       <c r="J144">
-        <v>40.53</v>
+        <v>18.62</v>
       </c>
       <c r="K144" t="s">
-        <v>270</v>
+        <v>677</v>
       </c>
       <c r="L144">
-        <v>9.1</v>
+        <v>14.39</v>
       </c>
       <c r="M144">
-        <v>2.07</v>
+        <v>27.85</v>
       </c>
       <c r="N144" t="s">
-        <v>335</v>
+        <v>734</v>
       </c>
     </row>
     <row r="145" spans="1:14">
@@ -19792,37 +19807,37 @@
         <v>17</v>
       </c>
       <c r="D145" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E145" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="F145">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G145" t="s">
-        <v>169</v>
+        <v>143</v>
       </c>
       <c r="H145">
-        <v>25.12</v>
+        <v>42.6</v>
       </c>
       <c r="I145" t="s">
-        <v>233</v>
+        <v>207</v>
       </c>
       <c r="J145">
-        <v>20.15</v>
+        <v>40.53</v>
       </c>
       <c r="K145" t="s">
-        <v>297</v>
+        <v>270</v>
       </c>
       <c r="L145">
-        <v>16.49</v>
+        <v>9.1</v>
       </c>
       <c r="M145">
-        <v>4.96</v>
+        <v>2.07</v>
       </c>
       <c r="N145" t="s">
-        <v>362</v>
+        <v>335</v>
       </c>
     </row>
     <row r="146" spans="1:14">
@@ -19836,37 +19851,37 @@
         <v>17</v>
       </c>
       <c r="D146" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E146" t="s">
-        <v>784</v>
+        <v>106</v>
       </c>
       <c r="F146">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G146" t="s">
-        <v>817</v>
+        <v>169</v>
       </c>
       <c r="H146">
-        <v>44.01</v>
+        <v>25.12</v>
       </c>
       <c r="I146" t="s">
-        <v>847</v>
+        <v>233</v>
       </c>
       <c r="J146">
-        <v>23.46</v>
+        <v>20.15</v>
       </c>
       <c r="K146" t="s">
-        <v>876</v>
+        <v>297</v>
       </c>
       <c r="L146">
-        <v>17.48</v>
+        <v>16.49</v>
       </c>
       <c r="M146">
-        <v>20.55</v>
+        <v>4.96</v>
       </c>
       <c r="N146" t="s">
-        <v>908</v>
+        <v>362</v>
       </c>
     </row>
     <row r="147" spans="1:14">
@@ -19880,37 +19895,37 @@
         <v>17</v>
       </c>
       <c r="D147" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="E147" t="s">
         <v>785</v>
       </c>
       <c r="F147">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G147" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="H147">
-        <v>48.23</v>
+        <v>44.01</v>
       </c>
       <c r="I147" t="s">
-        <v>824</v>
+        <v>850</v>
       </c>
       <c r="J147">
-        <v>35.75</v>
+        <v>23.46</v>
       </c>
       <c r="K147" t="s">
-        <v>877</v>
+        <v>880</v>
       </c>
       <c r="L147">
-        <v>16.02</v>
+        <v>17.48</v>
       </c>
       <c r="M147">
-        <v>12.48</v>
+        <v>20.55</v>
       </c>
       <c r="N147" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
     </row>
     <row r="148" spans="1:14">
@@ -19927,34 +19942,34 @@
         <v>21</v>
       </c>
       <c r="E148" t="s">
-        <v>381</v>
+        <v>786</v>
       </c>
       <c r="F148">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G148" t="s">
-        <v>405</v>
+        <v>820</v>
       </c>
       <c r="H148">
-        <v>36.77</v>
+        <v>48.23</v>
       </c>
       <c r="I148" t="s">
-        <v>427</v>
+        <v>826</v>
       </c>
       <c r="J148">
-        <v>25.34</v>
+        <v>35.75</v>
       </c>
       <c r="K148" t="s">
-        <v>448</v>
+        <v>881</v>
       </c>
       <c r="L148">
-        <v>24.32</v>
+        <v>16.02</v>
       </c>
       <c r="M148">
-        <v>11.43</v>
+        <v>12.48</v>
       </c>
       <c r="N148" t="s">
-        <v>470</v>
+        <v>914</v>
       </c>
     </row>
     <row r="149" spans="1:14">
@@ -19968,37 +19983,37 @@
         <v>17</v>
       </c>
       <c r="D149" t="s">
-        <v>760</v>
+        <v>21</v>
       </c>
       <c r="E149" t="s">
-        <v>786</v>
+        <v>381</v>
       </c>
       <c r="F149">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G149" t="s">
-        <v>819</v>
+        <v>405</v>
       </c>
       <c r="H149">
-        <v>45.42</v>
+        <v>36.77</v>
       </c>
       <c r="I149" t="s">
-        <v>848</v>
+        <v>427</v>
       </c>
       <c r="J149">
-        <v>38.94</v>
+        <v>25.34</v>
       </c>
       <c r="K149" t="s">
-        <v>878</v>
+        <v>448</v>
       </c>
       <c r="L149">
-        <v>15.64</v>
+        <v>24.32</v>
       </c>
       <c r="M149">
-        <v>6.49</v>
+        <v>11.43</v>
       </c>
       <c r="N149" t="s">
-        <v>910</v>
+        <v>470</v>
       </c>
     </row>
     <row r="150" spans="1:14">
@@ -20021,28 +20036,28 @@
         <v>3</v>
       </c>
       <c r="G150" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="H150">
-        <v>47.69</v>
+        <v>45.42</v>
       </c>
       <c r="I150" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="J150">
-        <v>28.08</v>
+        <v>38.94</v>
       </c>
       <c r="K150" t="s">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="L150">
-        <v>24.23</v>
+        <v>15.64</v>
       </c>
       <c r="M150">
-        <v>19.62</v>
+        <v>6.49</v>
       </c>
       <c r="N150" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
     </row>
     <row r="151" spans="1:14">
@@ -20056,37 +20071,37 @@
         <v>17</v>
       </c>
       <c r="D151" t="s">
-        <v>30</v>
+        <v>760</v>
       </c>
       <c r="E151" t="s">
         <v>788</v>
       </c>
       <c r="F151">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G151" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="H151">
-        <v>47.89</v>
+        <v>47.69</v>
       </c>
       <c r="I151" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
       <c r="J151">
-        <v>16.44</v>
+        <v>28.08</v>
       </c>
       <c r="K151" t="s">
-        <v>880</v>
+        <v>883</v>
       </c>
       <c r="L151">
-        <v>12.85</v>
+        <v>24.23</v>
       </c>
       <c r="M151">
-        <v>31.44</v>
+        <v>19.62</v>
       </c>
       <c r="N151" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
     </row>
     <row r="152" spans="1:14">
@@ -20100,37 +20115,37 @@
         <v>17</v>
       </c>
       <c r="D152" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E152" t="s">
-        <v>496</v>
+        <v>789</v>
       </c>
       <c r="F152">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G152" t="s">
-        <v>555</v>
+        <v>823</v>
       </c>
       <c r="H152">
-        <v>42.47</v>
+        <v>47.89</v>
       </c>
       <c r="I152" t="s">
-        <v>606</v>
+        <v>853</v>
       </c>
       <c r="J152">
-        <v>32.88</v>
+        <v>16.44</v>
       </c>
       <c r="K152" t="s">
-        <v>661</v>
+        <v>884</v>
       </c>
       <c r="L152">
-        <v>24.66</v>
+        <v>12.85</v>
       </c>
       <c r="M152">
-        <v>9.59</v>
+        <v>31.44</v>
       </c>
       <c r="N152" t="s">
-        <v>712</v>
+        <v>917</v>
       </c>
     </row>
     <row r="153" spans="1:14">
@@ -20144,37 +20159,37 @@
         <v>17</v>
       </c>
       <c r="D153" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="E153" t="s">
-        <v>59</v>
+        <v>496</v>
       </c>
       <c r="F153">
         <v>3</v>
       </c>
       <c r="G153" t="s">
-        <v>124</v>
+        <v>555</v>
       </c>
       <c r="H153">
-        <v>41.1</v>
+        <v>42.47</v>
       </c>
       <c r="I153" t="s">
-        <v>187</v>
+        <v>606</v>
       </c>
       <c r="J153">
-        <v>40.29</v>
+        <v>32.88</v>
       </c>
       <c r="K153" t="s">
-        <v>251</v>
+        <v>661</v>
       </c>
       <c r="L153">
-        <v>18.61</v>
+        <v>24.66</v>
       </c>
       <c r="M153">
-        <v>0.82</v>
+        <v>9.59</v>
       </c>
       <c r="N153" t="s">
-        <v>315</v>
+        <v>712</v>
       </c>
     </row>
     <row r="154" spans="1:14">
@@ -20191,34 +20206,34 @@
         <v>27</v>
       </c>
       <c r="E154" t="s">
-        <v>538</v>
+        <v>59</v>
       </c>
       <c r="F154">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G154" t="s">
-        <v>590</v>
+        <v>124</v>
       </c>
       <c r="H154">
-        <v>49.15</v>
+        <v>41.1</v>
       </c>
       <c r="I154" t="s">
-        <v>643</v>
+        <v>187</v>
       </c>
       <c r="J154">
-        <v>23.8</v>
+        <v>40.29</v>
       </c>
       <c r="K154" t="s">
-        <v>694</v>
+        <v>251</v>
       </c>
       <c r="L154">
-        <v>14.59</v>
+        <v>18.61</v>
       </c>
       <c r="M154">
-        <v>25.35</v>
+        <v>0.82</v>
       </c>
       <c r="N154" t="s">
-        <v>755</v>
+        <v>315</v>
       </c>
     </row>
     <row r="155" spans="1:14">
@@ -20232,42 +20247,42 @@
         <v>17</v>
       </c>
       <c r="D155" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E155" t="s">
-        <v>789</v>
+        <v>538</v>
       </c>
       <c r="F155">
         <v>4</v>
       </c>
       <c r="G155" t="s">
-        <v>822</v>
+        <v>590</v>
       </c>
       <c r="H155">
-        <v>42.37</v>
+        <v>49.15</v>
       </c>
       <c r="I155" t="s">
-        <v>851</v>
+        <v>643</v>
       </c>
       <c r="J155">
-        <v>22.21</v>
+        <v>23.8</v>
       </c>
       <c r="K155" t="s">
-        <v>881</v>
+        <v>694</v>
       </c>
       <c r="L155">
-        <v>21.98</v>
+        <v>14.59</v>
       </c>
       <c r="M155">
-        <v>20.16</v>
+        <v>25.35</v>
       </c>
       <c r="N155" t="s">
-        <v>913</v>
+        <v>755</v>
       </c>
     </row>
     <row r="156" spans="1:14">
       <c r="A156">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B156" t="s">
         <v>15</v>
@@ -20276,45 +20291,45 @@
         <v>17</v>
       </c>
       <c r="D156" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="E156" t="s">
         <v>790</v>
       </c>
       <c r="F156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G156" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="H156">
-        <v>44.68</v>
+        <v>42.37</v>
       </c>
       <c r="I156" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="J156">
-        <v>31</v>
+        <v>22.21</v>
       </c>
       <c r="K156" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="L156">
-        <v>24.32</v>
+        <v>21.98</v>
       </c>
       <c r="M156">
-        <v>13.68</v>
+        <v>20.16</v>
       </c>
       <c r="N156" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
     </row>
     <row r="157" spans="1:14">
       <c r="A157">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B157" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C157" t="s">
         <v>17</v>
@@ -20323,34 +20338,34 @@
         <v>25</v>
       </c>
       <c r="E157" t="s">
-        <v>53</v>
+        <v>791</v>
       </c>
       <c r="F157">
         <v>3</v>
       </c>
       <c r="G157" t="s">
-        <v>118</v>
+        <v>825</v>
       </c>
       <c r="H157">
-        <v>33.98</v>
+        <v>44.68</v>
       </c>
       <c r="I157" t="s">
-        <v>181</v>
+        <v>855</v>
       </c>
       <c r="J157">
-        <v>33.27</v>
+        <v>31</v>
       </c>
       <c r="K157" t="s">
-        <v>245</v>
+        <v>886</v>
       </c>
       <c r="L157">
-        <v>32.75</v>
+        <v>24.32</v>
       </c>
       <c r="M157">
-        <v>0.7</v>
+        <v>13.68</v>
       </c>
       <c r="N157" t="s">
-        <v>309</v>
+        <v>919</v>
       </c>
     </row>
     <row r="158" spans="1:14">
@@ -20358,43 +20373,43 @@
         <v>2025</v>
       </c>
       <c r="B158" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C158" t="s">
         <v>17</v>
       </c>
       <c r="D158" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E158" t="s">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="F158">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G158" t="s">
-        <v>160</v>
+        <v>118</v>
       </c>
       <c r="H158">
-        <v>28.77</v>
+        <v>33.98</v>
       </c>
       <c r="I158" t="s">
-        <v>225</v>
+        <v>181</v>
       </c>
       <c r="J158">
-        <v>24.73</v>
+        <v>33.27</v>
       </c>
       <c r="K158" t="s">
-        <v>288</v>
+        <v>245</v>
       </c>
       <c r="L158">
-        <v>16.1</v>
+        <v>32.75</v>
       </c>
       <c r="M158">
-        <v>4.04</v>
+        <v>0.7</v>
       </c>
       <c r="N158" t="s">
-        <v>353</v>
+        <v>309</v>
       </c>
     </row>
     <row r="159" spans="1:14">
@@ -20411,34 +20426,34 @@
         <v>24</v>
       </c>
       <c r="E159" t="s">
-        <v>485</v>
+        <v>97</v>
       </c>
       <c r="F159">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G159" t="s">
-        <v>545</v>
+        <v>160</v>
       </c>
       <c r="H159">
-        <v>39.11</v>
+        <v>28.77</v>
       </c>
       <c r="I159" t="s">
-        <v>596</v>
+        <v>225</v>
       </c>
       <c r="J159">
-        <v>33.52</v>
+        <v>24.73</v>
       </c>
       <c r="K159" t="s">
-        <v>650</v>
+        <v>288</v>
       </c>
       <c r="L159">
-        <v>27.37</v>
+        <v>16.1</v>
       </c>
       <c r="M159">
-        <v>5.58</v>
+        <v>4.04</v>
       </c>
       <c r="N159" t="s">
-        <v>701</v>
+        <v>353</v>
       </c>
     </row>
     <row r="160" spans="1:14">
@@ -20452,37 +20467,37 @@
         <v>17</v>
       </c>
       <c r="D160" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E160" t="s">
-        <v>520</v>
+        <v>485</v>
       </c>
       <c r="F160">
         <v>3</v>
       </c>
       <c r="G160" t="s">
-        <v>576</v>
+        <v>545</v>
       </c>
       <c r="H160">
-        <v>46.65</v>
+        <v>39.11</v>
       </c>
       <c r="I160" t="s">
-        <v>627</v>
+        <v>596</v>
       </c>
       <c r="J160">
-        <v>40.54</v>
+        <v>33.52</v>
       </c>
       <c r="K160" t="s">
-        <v>679</v>
+        <v>650</v>
       </c>
       <c r="L160">
-        <v>12.81</v>
+        <v>27.37</v>
       </c>
       <c r="M160">
-        <v>6.11</v>
+        <v>5.58</v>
       </c>
       <c r="N160" t="s">
-        <v>736</v>
+        <v>701</v>
       </c>
     </row>
     <row r="161" spans="1:14">
@@ -20496,37 +20511,37 @@
         <v>17</v>
       </c>
       <c r="D161" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E161" t="s">
-        <v>84</v>
+        <v>520</v>
       </c>
       <c r="F161">
         <v>3</v>
       </c>
       <c r="G161" t="s">
-        <v>148</v>
+        <v>576</v>
       </c>
       <c r="H161">
-        <v>38.28</v>
+        <v>46.65</v>
       </c>
       <c r="I161" t="s">
-        <v>212</v>
+        <v>627</v>
       </c>
       <c r="J161">
-        <v>35.71</v>
+        <v>40.54</v>
       </c>
       <c r="K161" t="s">
-        <v>275</v>
+        <v>679</v>
       </c>
       <c r="L161">
-        <v>26</v>
+        <v>12.81</v>
       </c>
       <c r="M161">
-        <v>2.57</v>
+        <v>6.11</v>
       </c>
       <c r="N161" t="s">
-        <v>340</v>
+        <v>736</v>
       </c>
     </row>
     <row r="162" spans="1:14">
@@ -20540,37 +20555,37 @@
         <v>17</v>
       </c>
       <c r="D162" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="E162" t="s">
-        <v>541</v>
+        <v>84</v>
       </c>
       <c r="F162">
         <v>3</v>
       </c>
       <c r="G162" t="s">
-        <v>593</v>
+        <v>148</v>
       </c>
       <c r="H162">
-        <v>49.79</v>
+        <v>38.28</v>
       </c>
       <c r="I162" t="s">
-        <v>646</v>
+        <v>212</v>
       </c>
       <c r="J162">
-        <v>39.88</v>
+        <v>35.71</v>
       </c>
       <c r="K162" t="s">
-        <v>697</v>
+        <v>275</v>
       </c>
       <c r="L162">
-        <v>10.12</v>
+        <v>26</v>
       </c>
       <c r="M162">
-        <v>9.92</v>
+        <v>2.57</v>
       </c>
       <c r="N162" t="s">
-        <v>758</v>
+        <v>340</v>
       </c>
     </row>
     <row r="163" spans="1:14">
@@ -20584,37 +20599,37 @@
         <v>17</v>
       </c>
       <c r="D163" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E163" t="s">
-        <v>378</v>
+        <v>541</v>
       </c>
       <c r="F163">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G163" t="s">
-        <v>402</v>
+        <v>593</v>
       </c>
       <c r="H163">
-        <v>36.39</v>
+        <v>49.79</v>
       </c>
       <c r="I163" t="s">
-        <v>424</v>
+        <v>646</v>
       </c>
       <c r="J163">
-        <v>21.95</v>
+        <v>39.88</v>
       </c>
       <c r="K163" t="s">
-        <v>445</v>
+        <v>697</v>
       </c>
       <c r="L163">
-        <v>20.1</v>
+        <v>10.12</v>
       </c>
       <c r="M163">
-        <v>14.44</v>
+        <v>9.92</v>
       </c>
       <c r="N163" t="s">
-        <v>467</v>
+        <v>758</v>
       </c>
     </row>
     <row r="164" spans="1:14">
@@ -20628,37 +20643,37 @@
         <v>17</v>
       </c>
       <c r="D164" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E164" t="s">
-        <v>61</v>
+        <v>378</v>
       </c>
       <c r="F164">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G164" t="s">
-        <v>580</v>
+        <v>402</v>
       </c>
       <c r="H164">
-        <v>47.16</v>
+        <v>36.39</v>
       </c>
       <c r="I164" t="s">
-        <v>632</v>
+        <v>424</v>
       </c>
       <c r="J164">
-        <v>34</v>
+        <v>21.95</v>
       </c>
       <c r="K164" t="s">
-        <v>683</v>
+        <v>445</v>
       </c>
       <c r="L164">
-        <v>18.84</v>
+        <v>20.1</v>
       </c>
       <c r="M164">
-        <v>13.16</v>
+        <v>14.44</v>
       </c>
       <c r="N164" t="s">
-        <v>742</v>
+        <v>467</v>
       </c>
     </row>
     <row r="165" spans="1:14">
@@ -20672,37 +20687,37 @@
         <v>17</v>
       </c>
       <c r="D165" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E165" t="s">
-        <v>482</v>
+        <v>61</v>
       </c>
       <c r="F165">
         <v>3</v>
       </c>
       <c r="G165" t="s">
-        <v>542</v>
+        <v>580</v>
       </c>
       <c r="H165">
-        <v>37.28</v>
+        <v>47.16</v>
       </c>
       <c r="I165" t="s">
-        <v>180</v>
+        <v>632</v>
       </c>
       <c r="J165">
-        <v>31.65</v>
+        <v>34</v>
       </c>
       <c r="K165" t="s">
-        <v>647</v>
+        <v>683</v>
       </c>
       <c r="L165">
-        <v>30.9</v>
+        <v>18.84</v>
       </c>
       <c r="M165">
-        <v>5.64</v>
+        <v>13.16</v>
       </c>
       <c r="N165" t="s">
-        <v>698</v>
+        <v>742</v>
       </c>
     </row>
     <row r="166" spans="1:14">
@@ -20716,37 +20731,37 @@
         <v>17</v>
       </c>
       <c r="D166" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E166" t="s">
-        <v>88</v>
+        <v>482</v>
       </c>
       <c r="F166">
         <v>3</v>
       </c>
       <c r="G166" t="s">
-        <v>152</v>
+        <v>542</v>
       </c>
       <c r="H166">
-        <v>41.93</v>
+        <v>37.28</v>
       </c>
       <c r="I166" t="s">
-        <v>216</v>
+        <v>180</v>
       </c>
       <c r="J166">
-        <v>39.15</v>
+        <v>31.65</v>
       </c>
       <c r="K166" t="s">
-        <v>279</v>
+        <v>647</v>
       </c>
       <c r="L166">
-        <v>18.93</v>
+        <v>30.9</v>
       </c>
       <c r="M166">
-        <v>2.78</v>
+        <v>5.64</v>
       </c>
       <c r="N166" t="s">
-        <v>344</v>
+        <v>698</v>
       </c>
     </row>
     <row r="167" spans="1:14">
@@ -20760,37 +20775,37 @@
         <v>17</v>
       </c>
       <c r="D167" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E167" t="s">
-        <v>507</v>
+        <v>88</v>
       </c>
       <c r="F167">
         <v>3</v>
       </c>
       <c r="G167" t="s">
-        <v>565</v>
+        <v>152</v>
       </c>
       <c r="H167">
-        <v>44.37</v>
+        <v>41.93</v>
       </c>
       <c r="I167" t="s">
-        <v>615</v>
+        <v>216</v>
       </c>
       <c r="J167">
-        <v>37.01</v>
+        <v>39.15</v>
       </c>
       <c r="K167" t="s">
-        <v>670</v>
+        <v>279</v>
       </c>
       <c r="L167">
-        <v>18.62</v>
+        <v>18.93</v>
       </c>
       <c r="M167">
-        <v>7.36</v>
+        <v>2.78</v>
       </c>
       <c r="N167" t="s">
-        <v>723</v>
+        <v>344</v>
       </c>
     </row>
     <row r="168" spans="1:14">
@@ -20804,37 +20819,37 @@
         <v>17</v>
       </c>
       <c r="D168" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E168" t="s">
-        <v>104</v>
+        <v>507</v>
       </c>
       <c r="F168">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G168" t="s">
-        <v>167</v>
+        <v>565</v>
       </c>
       <c r="H168">
-        <v>39.3</v>
+        <v>44.37</v>
       </c>
       <c r="I168" t="s">
-        <v>231</v>
+        <v>615</v>
       </c>
       <c r="J168">
-        <v>34.61</v>
+        <v>37.01</v>
       </c>
       <c r="K168" t="s">
-        <v>295</v>
+        <v>670</v>
       </c>
       <c r="L168">
-        <v>13.77</v>
+        <v>18.62</v>
       </c>
       <c r="M168">
-        <v>4.7</v>
+        <v>7.36</v>
       </c>
       <c r="N168" t="s">
-        <v>360</v>
+        <v>723</v>
       </c>
     </row>
     <row r="169" spans="1:14">
@@ -20848,37 +20863,37 @@
         <v>17</v>
       </c>
       <c r="D169" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E169" t="s">
-        <v>527</v>
+        <v>104</v>
       </c>
       <c r="F169">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G169" t="s">
-        <v>581</v>
+        <v>167</v>
       </c>
       <c r="H169">
-        <v>47.52</v>
+        <v>39.3</v>
       </c>
       <c r="I169" t="s">
-        <v>633</v>
+        <v>231</v>
       </c>
       <c r="J169">
-        <v>42.52</v>
+        <v>34.61</v>
       </c>
       <c r="K169" t="s">
-        <v>685</v>
+        <v>295</v>
       </c>
       <c r="L169">
-        <v>9.74</v>
+        <v>13.77</v>
       </c>
       <c r="M169">
-        <v>5.01</v>
+        <v>4.7</v>
       </c>
       <c r="N169" t="s">
-        <v>744</v>
+        <v>360</v>
       </c>
     </row>
     <row r="170" spans="1:14">
@@ -20892,37 +20907,37 @@
         <v>17</v>
       </c>
       <c r="D170" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="E170" t="s">
-        <v>74</v>
+        <v>527</v>
       </c>
       <c r="F170">
         <v>3</v>
       </c>
       <c r="G170" t="s">
-        <v>139</v>
+        <v>581</v>
       </c>
       <c r="H170">
-        <v>45.25</v>
+        <v>47.52</v>
       </c>
       <c r="I170" t="s">
-        <v>202</v>
+        <v>633</v>
       </c>
       <c r="J170">
-        <v>43.58</v>
+        <v>42.52</v>
       </c>
       <c r="K170" t="s">
-        <v>265</v>
+        <v>685</v>
       </c>
       <c r="L170">
-        <v>11.17</v>
+        <v>9.74</v>
       </c>
       <c r="M170">
-        <v>1.68</v>
+        <v>5.01</v>
       </c>
       <c r="N170" t="s">
-        <v>330</v>
+        <v>744</v>
       </c>
     </row>
     <row r="171" spans="1:14">
@@ -20939,34 +20954,34 @@
         <v>35</v>
       </c>
       <c r="E171" t="s">
-        <v>791</v>
+        <v>74</v>
       </c>
       <c r="F171">
         <v>3</v>
       </c>
       <c r="G171" t="s">
-        <v>396</v>
+        <v>139</v>
       </c>
       <c r="H171">
-        <v>45.69</v>
+        <v>45.25</v>
       </c>
       <c r="I171" t="s">
-        <v>853</v>
+        <v>202</v>
       </c>
       <c r="J171">
-        <v>32.91</v>
+        <v>43.58</v>
       </c>
       <c r="K171" t="s">
-        <v>439</v>
+        <v>265</v>
       </c>
       <c r="L171">
-        <v>21.39</v>
+        <v>11.17</v>
       </c>
       <c r="M171">
-        <v>12.78</v>
+        <v>1.68</v>
       </c>
       <c r="N171" t="s">
-        <v>915</v>
+        <v>330</v>
       </c>
     </row>
     <row r="172" spans="1:14">
@@ -20980,7 +20995,7 @@
         <v>17</v>
       </c>
       <c r="D172" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E172" t="s">
         <v>792</v>
@@ -20989,28 +21004,28 @@
         <v>3</v>
       </c>
       <c r="G172" t="s">
-        <v>824</v>
+        <v>396</v>
       </c>
       <c r="H172">
-        <v>47.83</v>
+        <v>45.69</v>
       </c>
       <c r="I172" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="J172">
-        <v>29.17</v>
+        <v>32.91</v>
       </c>
       <c r="K172" t="s">
-        <v>883</v>
+        <v>439</v>
       </c>
       <c r="L172">
-        <v>23</v>
+        <v>21.39</v>
       </c>
       <c r="M172">
-        <v>18.67</v>
+        <v>12.78</v>
       </c>
       <c r="N172" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
     </row>
     <row r="173" spans="1:14">
@@ -21024,7 +21039,7 @@
         <v>17</v>
       </c>
       <c r="D173" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E173" t="s">
         <v>793</v>
@@ -21033,28 +21048,28 @@
         <v>3</v>
       </c>
       <c r="G173" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="H173">
-        <v>45.5</v>
+        <v>47.83</v>
       </c>
       <c r="I173" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
       <c r="J173">
-        <v>27.7</v>
+        <v>29.17</v>
       </c>
       <c r="K173" t="s">
-        <v>884</v>
+        <v>887</v>
       </c>
       <c r="L173">
-        <v>26.8</v>
+        <v>23</v>
       </c>
       <c r="M173">
-        <v>17.81</v>
+        <v>18.67</v>
       </c>
       <c r="N173" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
     </row>
     <row r="174" spans="1:14">
@@ -21068,37 +21083,37 @@
         <v>17</v>
       </c>
       <c r="D174" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E174" t="s">
-        <v>54</v>
+        <v>794</v>
       </c>
       <c r="F174">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G174" t="s">
-        <v>119</v>
+        <v>827</v>
       </c>
       <c r="H174">
-        <v>38.72</v>
+        <v>45.5</v>
       </c>
       <c r="I174" t="s">
-        <v>182</v>
+        <v>858</v>
       </c>
       <c r="J174">
-        <v>38</v>
+        <v>27.7</v>
       </c>
       <c r="K174" t="s">
-        <v>246</v>
+        <v>888</v>
       </c>
       <c r="L174">
+        <v>26.8</v>
+      </c>
+      <c r="M174">
         <v>17.81</v>
       </c>
-      <c r="M174">
-        <v>0.71</v>
-      </c>
       <c r="N174" t="s">
-        <v>310</v>
+        <v>922</v>
       </c>
     </row>
     <row r="175" spans="1:14">
@@ -21112,37 +21127,37 @@
         <v>17</v>
       </c>
       <c r="D175" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="E175" t="s">
-        <v>531</v>
+        <v>54</v>
       </c>
       <c r="F175">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G175" t="s">
-        <v>584</v>
+        <v>119</v>
       </c>
       <c r="H175">
-        <v>48</v>
+        <v>38.72</v>
       </c>
       <c r="I175" t="s">
-        <v>637</v>
+        <v>182</v>
       </c>
       <c r="J175">
-        <v>40.62</v>
+        <v>38</v>
       </c>
       <c r="K175" t="s">
-        <v>688</v>
+        <v>246</v>
       </c>
       <c r="L175">
-        <v>11.38</v>
+        <v>17.81</v>
       </c>
       <c r="M175">
-        <v>7.38</v>
+        <v>0.71</v>
       </c>
       <c r="N175" t="s">
-        <v>748</v>
+        <v>310</v>
       </c>
     </row>
     <row r="176" spans="1:14">
@@ -21156,37 +21171,37 @@
         <v>17</v>
       </c>
       <c r="D176" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="E176" t="s">
-        <v>375</v>
+        <v>531</v>
       </c>
       <c r="F176">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G176" t="s">
-        <v>400</v>
+        <v>584</v>
       </c>
       <c r="H176">
-        <v>35.37</v>
+        <v>48</v>
       </c>
       <c r="I176" t="s">
-        <v>422</v>
+        <v>637</v>
       </c>
       <c r="J176">
-        <v>26.87</v>
+        <v>40.62</v>
       </c>
       <c r="K176" t="s">
-        <v>443</v>
+        <v>688</v>
       </c>
       <c r="L176">
-        <v>26.53</v>
+        <v>11.38</v>
       </c>
       <c r="M176">
-        <v>8.5</v>
+        <v>7.38</v>
       </c>
       <c r="N176" t="s">
-        <v>464</v>
+        <v>748</v>
       </c>
     </row>
     <row r="177" spans="1:14">
@@ -21200,37 +21215,37 @@
         <v>17</v>
       </c>
       <c r="D177" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E177" t="s">
-        <v>499</v>
+        <v>375</v>
       </c>
       <c r="F177">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G177" t="s">
-        <v>557</v>
+        <v>400</v>
       </c>
       <c r="H177">
-        <v>42.99</v>
+        <v>35.37</v>
       </c>
       <c r="I177" t="s">
-        <v>608</v>
+        <v>422</v>
       </c>
       <c r="J177">
-        <v>34.85</v>
+        <v>26.87</v>
       </c>
       <c r="K177" t="s">
-        <v>663</v>
+        <v>443</v>
       </c>
       <c r="L177">
-        <v>22.16</v>
+        <v>26.53</v>
       </c>
       <c r="M177">
-        <v>8.140000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="N177" t="s">
-        <v>715</v>
+        <v>464</v>
       </c>
     </row>
     <row r="178" spans="1:14">
@@ -21247,34 +21262,34 @@
         <v>30</v>
       </c>
       <c r="E178" t="s">
-        <v>66</v>
+        <v>499</v>
       </c>
       <c r="F178">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G178" t="s">
-        <v>131</v>
+        <v>557</v>
       </c>
       <c r="H178">
-        <v>28.21</v>
+        <v>42.99</v>
       </c>
       <c r="I178" t="s">
-        <v>194</v>
+        <v>608</v>
       </c>
       <c r="J178">
-        <v>26.83</v>
+        <v>34.85</v>
       </c>
       <c r="K178" t="s">
-        <v>257</v>
+        <v>663</v>
       </c>
       <c r="L178">
-        <v>24.31</v>
+        <v>22.16</v>
       </c>
       <c r="M178">
-        <v>1.38</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N178" t="s">
-        <v>322</v>
+        <v>715</v>
       </c>
     </row>
     <row r="179" spans="1:14">
@@ -21291,34 +21306,34 @@
         <v>30</v>
       </c>
       <c r="E179" t="s">
-        <v>509</v>
+        <v>66</v>
       </c>
       <c r="F179">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G179" t="s">
-        <v>567</v>
+        <v>131</v>
       </c>
       <c r="H179">
-        <v>45.03</v>
+        <v>28.21</v>
       </c>
       <c r="I179" t="s">
-        <v>617</v>
+        <v>194</v>
       </c>
       <c r="J179">
-        <v>37.41</v>
+        <v>26.83</v>
       </c>
       <c r="K179" t="s">
-        <v>671</v>
+        <v>257</v>
       </c>
       <c r="L179">
-        <v>17.55</v>
+        <v>24.31</v>
       </c>
       <c r="M179">
-        <v>7.62</v>
+        <v>1.38</v>
       </c>
       <c r="N179" t="s">
-        <v>725</v>
+        <v>322</v>
       </c>
     </row>
     <row r="180" spans="1:14">
@@ -21332,37 +21347,37 @@
         <v>17</v>
       </c>
       <c r="D180" t="s">
-        <v>366</v>
+        <v>30</v>
       </c>
       <c r="E180" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="F180">
         <v>3</v>
       </c>
       <c r="G180" t="s">
-        <v>558</v>
+        <v>567</v>
       </c>
       <c r="H180">
-        <v>43.09</v>
+        <v>45.03</v>
       </c>
       <c r="I180" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="J180">
-        <v>33.79</v>
+        <v>37.41</v>
       </c>
       <c r="K180" t="s">
-        <v>664</v>
+        <v>671</v>
       </c>
       <c r="L180">
-        <v>23.12</v>
+        <v>17.55</v>
       </c>
       <c r="M180">
-        <v>9.300000000000001</v>
+        <v>7.62</v>
       </c>
       <c r="N180" t="s">
-        <v>716</v>
+        <v>725</v>
       </c>
     </row>
     <row r="181" spans="1:14">
@@ -21376,37 +21391,37 @@
         <v>17</v>
       </c>
       <c r="D181" t="s">
-        <v>32</v>
+        <v>366</v>
       </c>
       <c r="E181" t="s">
-        <v>91</v>
+        <v>500</v>
       </c>
       <c r="F181">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G181" t="s">
-        <v>155</v>
+        <v>558</v>
       </c>
       <c r="H181">
-        <v>29.84</v>
+        <v>43.09</v>
       </c>
       <c r="I181" t="s">
-        <v>219</v>
+        <v>609</v>
       </c>
       <c r="J181">
-        <v>26.47</v>
+        <v>33.79</v>
       </c>
       <c r="K181" t="s">
-        <v>282</v>
+        <v>664</v>
       </c>
       <c r="L181">
-        <v>21.98</v>
+        <v>23.12</v>
       </c>
       <c r="M181">
-        <v>3.37</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="N181" t="s">
-        <v>347</v>
+        <v>716</v>
       </c>
     </row>
     <row r="182" spans="1:14">
@@ -21423,34 +21438,34 @@
         <v>32</v>
       </c>
       <c r="E182" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="F182">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G182" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="H182">
-        <v>39.85</v>
+        <v>29.84</v>
       </c>
       <c r="I182" t="s">
-        <v>199</v>
+        <v>219</v>
       </c>
       <c r="J182">
-        <v>38.3</v>
+        <v>26.47</v>
       </c>
       <c r="K182" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="L182">
-        <v>21.85</v>
+        <v>21.98</v>
       </c>
       <c r="M182">
-        <v>1.54</v>
+        <v>3.37</v>
       </c>
       <c r="N182" t="s">
-        <v>327</v>
+        <v>347</v>
       </c>
     </row>
     <row r="183" spans="1:14">
@@ -21467,80 +21482,83 @@
         <v>32</v>
       </c>
       <c r="E183" t="s">
+        <v>71</v>
+      </c>
+      <c r="F183">
+        <v>3</v>
+      </c>
+      <c r="G183" t="s">
+        <v>136</v>
+      </c>
+      <c r="H183">
+        <v>39.85</v>
+      </c>
+      <c r="I183" t="s">
+        <v>199</v>
+      </c>
+      <c r="J183">
+        <v>38.3</v>
+      </c>
+      <c r="K183" t="s">
+        <v>262</v>
+      </c>
+      <c r="L183">
+        <v>21.85</v>
+      </c>
+      <c r="M183">
+        <v>1.54</v>
+      </c>
+      <c r="N183" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14">
+      <c r="A184">
+        <v>2025</v>
+      </c>
+      <c r="B184" t="s">
+        <v>15</v>
+      </c>
+      <c r="C184" t="s">
+        <v>17</v>
+      </c>
+      <c r="D184" t="s">
+        <v>32</v>
+      </c>
+      <c r="E184" t="s">
         <v>78</v>
       </c>
-      <c r="F183">
+      <c r="F184">
         <v>4</v>
       </c>
-      <c r="G183" t="s">
+      <c r="G184" t="s">
         <v>142</v>
       </c>
-      <c r="H183">
+      <c r="H184">
         <v>37.27</v>
       </c>
-      <c r="I183" t="s">
+      <c r="I184" t="s">
         <v>206</v>
       </c>
-      <c r="J183">
+      <c r="J184">
         <v>35.23</v>
       </c>
-      <c r="K183" t="s">
+      <c r="K184" t="s">
         <v>269</v>
       </c>
-      <c r="L183">
+      <c r="L184">
         <v>14.43</v>
       </c>
-      <c r="M183">
+      <c r="M184">
         <v>2.05</v>
       </c>
-      <c r="N183" t="s">
+      <c r="N184" t="s">
         <v>334</v>
-      </c>
-    </row>
-    <row r="184" spans="1:14">
-      <c r="A184" t="s">
-        <v>364</v>
-      </c>
-      <c r="B184" t="s">
-        <v>15</v>
-      </c>
-      <c r="C184" t="s">
-        <v>365</v>
-      </c>
-      <c r="E184" t="s">
-        <v>379</v>
-      </c>
-      <c r="F184">
-        <v>5</v>
-      </c>
-      <c r="G184" t="s">
-        <v>403</v>
-      </c>
-      <c r="H184">
-        <v>36.64</v>
-      </c>
-      <c r="I184" t="s">
-        <v>425</v>
-      </c>
-      <c r="J184">
-        <v>24.61</v>
-      </c>
-      <c r="K184" t="s">
-        <v>446</v>
-      </c>
-      <c r="L184">
-        <v>15.26</v>
-      </c>
-      <c r="M184">
-        <v>12.03</v>
-      </c>
-      <c r="N184" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="185" spans="1:14">
       <c r="A185" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B185" t="s">
         <v>15</v>
@@ -21549,33 +21567,74 @@
         <v>365</v>
       </c>
       <c r="E185" t="s">
+        <v>379</v>
+      </c>
+      <c r="F185">
+        <v>5</v>
+      </c>
+      <c r="G185" t="s">
+        <v>403</v>
+      </c>
+      <c r="H185">
+        <v>36.64</v>
+      </c>
+      <c r="I185" t="s">
+        <v>425</v>
+      </c>
+      <c r="J185">
+        <v>24.61</v>
+      </c>
+      <c r="K185" t="s">
+        <v>446</v>
+      </c>
+      <c r="L185">
+        <v>15.26</v>
+      </c>
+      <c r="M185">
+        <v>12.03</v>
+      </c>
+      <c r="N185" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="186" spans="1:14">
+      <c r="A186" t="s">
+        <v>363</v>
+      </c>
+      <c r="B186" t="s">
+        <v>15</v>
+      </c>
+      <c r="C186" t="s">
+        <v>365</v>
+      </c>
+      <c r="E186" t="s">
         <v>370</v>
       </c>
-      <c r="F185">
+      <c r="F186">
         <v>6</v>
       </c>
-      <c r="G185" t="s">
+      <c r="G186" t="s">
         <v>395</v>
       </c>
-      <c r="H185">
+      <c r="H186">
         <v>32.65</v>
       </c>
-      <c r="I185" t="s">
+      <c r="I186" t="s">
         <v>417</v>
       </c>
-      <c r="J185">
+      <c r="J186">
         <v>22.78</v>
       </c>
-      <c r="K185" t="s">
+      <c r="K186" t="s">
         <v>438</v>
       </c>
-      <c r="L185">
+      <c r="L186">
         <v>22.03</v>
       </c>
-      <c r="M185">
+      <c r="M186">
         <v>9.869999999999999</v>
       </c>
-      <c r="N185" t="s">
+      <c r="N186" t="s">
         <v>459</v>
       </c>
     </row>

</xml_diff>